<commit_message>
Added Exercise 4A SQL File
</commit_message>
<xml_diff>
--- a/Melgara_Ex3A_tables.xlsx
+++ b/Melgara_Ex3A_tables.xlsx
@@ -5,17 +5,17 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\smayamelgara\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\smayamelgara\Documents\DATA_Labs\W2_Workshop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A2966C7-EFCB-47E9-A37B-929E3378FFA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2934D454-FF0B-4E63-BCF7-BEB8B34AD548}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11964" yWindow="444" windowWidth="10896" windowHeight="8616" xr2:uid="{6A39D6D0-7092-4ABE-87E7-0C9BE5350AF7}"/>
+    <workbookView xWindow="6756" yWindow="1572" windowWidth="10896" windowHeight="8616" firstSheet="3" activeTab="3" xr2:uid="{6A39D6D0-7092-4ABE-87E7-0C9BE5350AF7}"/>
   </bookViews>
   <sheets>
     <sheet name="Customer_Data" sheetId="1" r:id="rId1"/>
     <sheet name="Dog_Data" sheetId="2" r:id="rId2"/>
-    <sheet name="Appointments_Data" sheetId="3" r:id="rId3"/>
+    <sheet name="Appointment_Data" sheetId="3" r:id="rId3"/>
     <sheet name="Payments_Data" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>

</xml_diff>